<commit_message>
Fix #12728 - [Bug] Update Citeo export report file
</commit_message>
<xml_diff>
--- a/becpg-plm/becpg-plm-core/src/main/resources/beCPG/birt/exportsearch/product/en/ExportCiteo.xlsx
+++ b/becpg-plm/becpg-plm-core/src/main/resources/beCPG/birt/exportsearch/product/en/ExportCiteo.xlsx
@@ -12,8 +12,8 @@
     <sheet name="Materials" sheetId="2" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">Materials!$B$3:$H$3</definedName>
-    <definedName function="false" hidden="false" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">Materials!$B$3:$H$4</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">Materials!$B$3:$H$4</definedName>
+    <definedName function="false" hidden="false" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">Materials!$B$3:$H$3</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="109">
   <si>
     <t xml:space="preserve">TYPE</t>
   </si>
@@ -186,13 +186,13 @@
     <t xml:space="preserve">Name</t>
   </si>
   <si>
-    <t xml:space="preserve">Commercial label</t>
+    <t xml:space="preserve">Trade name</t>
   </si>
   <si>
     <t xml:space="preserve">Label</t>
   </si>
   <si>
-    <t xml:space="preserve">BeCPG Code</t>
+    <t xml:space="preserve">beCPG Code</t>
   </si>
   <si>
     <t xml:space="preserve">ERP Code</t>
@@ -201,7 +201,7 @@
     <t xml:space="preserve">Product Code</t>
   </si>
   <si>
-    <t xml:space="preserve">Legal label</t>
+    <t xml:space="preserve">Legal name</t>
   </si>
   <si>
     <t xml:space="preserve">Number of packaging units on the product
@@ -299,6 +299,39 @@
   </si>
   <si>
     <t xml:space="preserve">Total per line</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6.1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6.2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6 .6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6.3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6.5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6.6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6.4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6.7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7.1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7.2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7.3</t>
   </si>
   <si>
     <t xml:space="preserve">pack:packMaterialList</t>
@@ -428,7 +461,7 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="14">
+  <fills count="15">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -474,7 +507,7 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFDDDDDD"/>
-        <bgColor rgb="FFF7C7CD"/>
+        <bgColor rgb="FFEEEEEE"/>
       </patternFill>
     </fill>
     <fill>
@@ -499,6 +532,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFF7C7CD"/>
         <bgColor rgb="FFDDDDDD"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFEEEEEE"/>
+        <bgColor rgb="FFFFFFFF"/>
       </patternFill>
     </fill>
     <fill>
@@ -603,7 +642,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="22">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -676,15 +715,19 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="true"/>
     </xf>
+    <xf numFmtId="164" fontId="8" fillId="13" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="13" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="14" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="11" fillId="13" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="11" fillId="14" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -717,7 +760,7 @@
       <rgbColor rgb="FF808080"/>
       <rgbColor rgb="FF9999FF"/>
       <rgbColor rgb="FF993366"/>
-      <rgbColor rgb="FFF7C7CD"/>
+      <rgbColor rgb="FFEEEEEE"/>
       <rgbColor rgb="FFCCFFFF"/>
       <rgbColor rgb="FF660066"/>
       <rgbColor rgb="FFED7483"/>
@@ -737,7 +780,7 @@
       <rgbColor rgb="FFFFFF99"/>
       <rgbColor rgb="FF80CEF4"/>
       <rgbColor rgb="FFF2987A"/>
-      <rgbColor rgb="FFCC99FF"/>
+      <rgbColor rgb="FFF7C7CD"/>
       <rgbColor rgb="FFFDD17A"/>
       <rgbColor rgb="FF3366FF"/>
       <rgbColor rgb="FF33CCCC"/>
@@ -767,13 +810,13 @@
       <xdr:col>34</xdr:col>
       <xdr:colOff>245880</xdr:colOff>
       <xdr:row>2</xdr:row>
-      <xdr:rowOff>62280</xdr:rowOff>
+      <xdr:rowOff>62640</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>34</xdr:col>
-      <xdr:colOff>389160</xdr:colOff>
+      <xdr:colOff>388080</xdr:colOff>
       <xdr:row>2</xdr:row>
-      <xdr:rowOff>62640</xdr:rowOff>
+      <xdr:rowOff>63000</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -782,8 +825,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="27924120" y="527400"/>
-          <a:ext cx="143280" cy="360"/>
+          <a:off x="28053720" y="527760"/>
+          <a:ext cx="142200" cy="360"/>
         </a:xfrm>
         <a:prstGeom prst="rightArrow">
           <a:avLst>
@@ -857,13 +900,13 @@
       <xdr:col>34</xdr:col>
       <xdr:colOff>245880</xdr:colOff>
       <xdr:row>2</xdr:row>
-      <xdr:rowOff>62280</xdr:rowOff>
+      <xdr:rowOff>62640</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>34</xdr:col>
-      <xdr:colOff>389160</xdr:colOff>
+      <xdr:colOff>388080</xdr:colOff>
       <xdr:row>2</xdr:row>
-      <xdr:rowOff>62640</xdr:rowOff>
+      <xdr:rowOff>63000</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -872,8 +915,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="27924120" y="527400"/>
-          <a:ext cx="143280" cy="360"/>
+          <a:off x="28053720" y="527760"/>
+          <a:ext cx="142200" cy="360"/>
         </a:xfrm>
         <a:prstGeom prst="rightArrow">
           <a:avLst>
@@ -947,13 +990,13 @@
       <xdr:col>34</xdr:col>
       <xdr:colOff>245880</xdr:colOff>
       <xdr:row>2</xdr:row>
-      <xdr:rowOff>62280</xdr:rowOff>
+      <xdr:rowOff>62640</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>34</xdr:col>
-      <xdr:colOff>389160</xdr:colOff>
+      <xdr:colOff>388080</xdr:colOff>
       <xdr:row>2</xdr:row>
-      <xdr:rowOff>62640</xdr:rowOff>
+      <xdr:rowOff>63000</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -962,8 +1005,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="27924120" y="527400"/>
-          <a:ext cx="143280" cy="360"/>
+          <a:off x="28053720" y="527760"/>
+          <a:ext cx="142200" cy="360"/>
         </a:xfrm>
         <a:prstGeom prst="rightArrow">
           <a:avLst>
@@ -1037,13 +1080,13 @@
       <xdr:col>34</xdr:col>
       <xdr:colOff>245880</xdr:colOff>
       <xdr:row>2</xdr:row>
-      <xdr:rowOff>62280</xdr:rowOff>
+      <xdr:rowOff>62640</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>34</xdr:col>
-      <xdr:colOff>389160</xdr:colOff>
+      <xdr:colOff>388080</xdr:colOff>
       <xdr:row>2</xdr:row>
-      <xdr:rowOff>62640</xdr:rowOff>
+      <xdr:rowOff>63000</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -1052,8 +1095,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="27924120" y="527400"/>
-          <a:ext cx="143280" cy="360"/>
+          <a:off x="28053720" y="527760"/>
+          <a:ext cx="142200" cy="360"/>
         </a:xfrm>
         <a:prstGeom prst="rightArrow">
           <a:avLst>
@@ -1134,8 +1177,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:AN6"/>
-  <sheetFormatPr defaultColWidth="11.55078125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:AN7"/>
+  <sheetFormatPr defaultColWidth="11.60546875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -1518,6 +1561,62 @@
       </c>
       <c r="AN6" s="13" t="s">
         <v>84</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="12.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="K7" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="L7" s="18" t="n">
+        <v>2</v>
+      </c>
+      <c r="M7" s="18" t="n">
+        <v>3</v>
+      </c>
+      <c r="N7" s="18" t="n">
+        <v>4</v>
+      </c>
+      <c r="O7" s="18" t="n">
+        <v>5</v>
+      </c>
+      <c r="P7" s="18" t="s">
+        <v>85</v>
+      </c>
+      <c r="Q7" s="18" t="s">
+        <v>86</v>
+      </c>
+      <c r="R7" s="18" t="s">
+        <v>87</v>
+      </c>
+      <c r="S7" s="18" t="s">
+        <v>88</v>
+      </c>
+      <c r="T7" s="18" t="s">
+        <v>89</v>
+      </c>
+      <c r="U7" s="18" t="s">
+        <v>90</v>
+      </c>
+      <c r="V7" s="18" t="s">
+        <v>91</v>
+      </c>
+      <c r="W7" s="18" t="s">
+        <v>90</v>
+      </c>
+      <c r="X7" s="18" t="s">
+        <v>92</v>
+      </c>
+      <c r="Y7" s="18" t="s">
+        <v>93</v>
+      </c>
+      <c r="Z7" s="18" t="s">
+        <v>94</v>
+      </c>
+      <c r="AA7" s="18" t="s">
+        <v>95</v>
       </c>
     </row>
   </sheetData>
@@ -1573,12 +1672,12 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:H3"/>
-  <sheetFormatPr defaultColWidth="8.42578125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.453125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="1" min="1" style="0" width="11.52"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="15.53"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="4" style="0" width="10.65"/>
-    <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="6" min="6" style="0" width="11.52"/>
+    <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="1" min="1" style="2" width="11.52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="2" width="15.53"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="4" style="2" width="10.65"/>
+    <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="6" min="6" style="2" width="11.52"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1586,12 +1685,8 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
+        <v>96</v>
+      </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
@@ -1601,52 +1696,52 @@
         <v>6</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="D2" s="18" t="s">
-        <v>87</v>
-      </c>
-      <c r="E2" s="18" t="s">
-        <v>88</v>
-      </c>
-      <c r="F2" s="18" t="s">
-        <v>89</v>
+        <v>97</v>
+      </c>
+      <c r="D2" s="19" t="s">
+        <v>98</v>
+      </c>
+      <c r="E2" s="19" t="s">
+        <v>99</v>
+      </c>
+      <c r="F2" s="19" t="s">
+        <v>100</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>90</v>
-      </c>
-      <c r="H2" s="0" t="s">
-        <v>91</v>
+        <v>101</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>102</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="B3" s="19" t="s">
-        <v>92</v>
-      </c>
-      <c r="C3" s="19" t="s">
+      <c r="B3" s="20" t="s">
+        <v>103</v>
+      </c>
+      <c r="C3" s="20" t="s">
         <v>46</v>
       </c>
-      <c r="D3" s="20" t="s">
-        <v>93</v>
-      </c>
-      <c r="E3" s="20" t="s">
-        <v>94</v>
-      </c>
-      <c r="F3" s="20" t="s">
-        <v>95</v>
-      </c>
-      <c r="G3" s="19" t="s">
-        <v>96</v>
-      </c>
-      <c r="H3" s="19" t="s">
-        <v>97</v>
+      <c r="D3" s="21" t="s">
+        <v>104</v>
+      </c>
+      <c r="E3" s="21" t="s">
+        <v>105</v>
+      </c>
+      <c r="F3" s="21" t="s">
+        <v>106</v>
+      </c>
+      <c r="G3" s="20" t="s">
+        <v>107</v>
+      </c>
+      <c r="H3" s="20" t="s">
+        <v>108</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="B3:H3"/>
+  <autoFilter ref="B3:H4"/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
   <pageSetup paperSize="9" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>

</xml_diff>